<commit_message>
Add ep10 summary: battery charge status monitor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LVeNQCCauU1jD51BpjCme9
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -903,23 +903,91 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="21">
-      <c r="A7" s="30" t="n"/>
-      <c r="B7" s="30" t="n"/>
-      <c r="C7" s="30" t="n"/>
-      <c r="D7" s="30" t="n"/>
-      <c r="E7" s="31" t="n"/>
-      <c r="F7" s="30" t="n"/>
-      <c r="G7" s="30" t="n"/>
-      <c r="H7" s="30" t="n"/>
-      <c r="I7" s="30" t="n"/>
-      <c r="J7" s="30" t="n"/>
-      <c r="K7" s="30" t="n"/>
-      <c r="L7" s="30" t="n"/>
-      <c r="M7" s="30" t="n"/>
-      <c r="N7" s="30" t="n"/>
-      <c r="O7" s="30" t="n"/>
-      <c r="P7" s="30" t="n"/>
+    <row r="7" ht="165" customHeight="1" s="21">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>Professional Electronic Design Course</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Designing a battery charge status monitoring circuit</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>Open README</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>Watch video</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>• Saturated transistor pulls its collector to ≈ 0 V (12 V / 0 V output)
+• Inverting transistor pair: Q1 on → Q2 off, Q1 off → Q2 on
+• Zener in the base path as a voltage-level detector
+• Designing resistor values from β_min, saturation factor and I_Z,min</t>
+        </is>
+      </c>
+      <c r="I7" s="25" t="inlineStr">
+        <is>
+          <t>1. Transistor switch with 10 kΩ collector load (12 V / 0 V demo)
+2. Inverting pair with green/red LEDs driven by a push switch
+3. Battery monitor: 10 V Zener replaces the switch (green ≥ 10 V, red &lt; 10 V)</t>
+        </is>
+      </c>
+      <c r="J7" s="25" t="inlineStr">
+        <is>
+          <t>I_B = I_C / β_min = 10 mA / 200 = 50 µA
+I_B1 = 10 × 50 µA = 0.5 mA
+11 − V_Z − I_B1·R_B1 − 0.7 = 0 → R_B1 ≈ 600 Ω
+10 − 0.7 = I_B2(1 kΩ + R_B2), I_B2 = 200 µA → R_B2 ≈ 46 kΩ</t>
+        </is>
+      </c>
+      <c r="K7" s="25" t="inlineStr">
+        <is>
+          <t>2 × BC547B (β 200–450), BZX85C10 Zener (9.4–10.6 V), R_B1 = 677 Ω (600 Ω calc, 10 kΩ also works), R_B2 = 46 kΩ, 2 × 1 kΩ, red + green LED, 12 V battery</t>
+        </is>
+      </c>
+      <c r="L7" s="25" t="inlineStr">
+        <is>
+          <t>Not simulated yet</t>
+        </is>
+      </c>
+      <c r="M7" s="25" t="inlineStr">
+        <is>
+          <t>12 V, 11 V → green ✔; ≤ 10 V → red ✔; switch point ≈ 10.5 V (red starts glowing ≈ 10.6 V). With R_B1 = 10 kΩ still switches between 10 V and 11 V, lower battery drain.</t>
+        </is>
+      </c>
+      <c r="N7" s="25" t="inlineStr">
+        <is>
+          <t>README only (no media yet)</t>
+        </is>
+      </c>
+      <c r="O7" s="25" t="inlineStr">
+        <is>
+          <t>Adding one Zener to an inverting transistor pair turns it into a voltage monitor; swap the Zener for an LDR or thermistor and it becomes a light or temperature indicator. Calculated values are a starting point, then adjust by testing.</t>
+        </is>
+      </c>
+      <c r="P7" s="25" t="inlineStr">
+        <is>
+          <t>To do: Circuit Wizard sim sweeping 12 → 9 V to find my switch point; try R_B1 = 677 Ω vs 10 kΩ; try an LDR version (light/dark indicator).</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="21">
       <c r="A8" s="30" t="n"/>
@@ -1532,6 +1600,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" display="Watch video" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add ep10 simulation video: battery voltage sweep
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LVeNQCCauU1jD51BpjCme9
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -919,7 +919,7 @@
       </c>
       <c r="D7" s="27" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" s="28" t="n">
@@ -965,7 +965,9 @@
       </c>
       <c r="L7" s="25" t="inlineStr">
         <is>
-          <t>Not simulated yet</t>
+          <t>• R_B1 = 10 kΩ: 11 V → green, I_B1 = 52 µA, V_CE(Q1) = 101 mV ✔; 10 V → red 2.12 V, Zener 9.56 V at 0 A ✔; 8 V → red ✔
+• R_B1 = 677 Ω: 11 V → green, I_B1 = 638 µA, V_CE(Q1) = 24 mV ✔; 10 V → red ✔; 5 V → red dim
+• ≤ 3 V → neither LED lights</t>
         </is>
       </c>
       <c r="M7" s="25" t="inlineStr">
@@ -975,7 +977,7 @@
       </c>
       <c r="N7" s="25" t="inlineStr">
         <is>
-          <t>README only (no media yet)</t>
+          <t>1 simulation GIF + MP4: battery voltage sweep (10 kΩ vs 677 Ω)</t>
         </is>
       </c>
       <c r="O7" s="25" t="inlineStr">
@@ -985,7 +987,7 @@
       </c>
       <c r="P7" s="25" t="inlineStr">
         <is>
-          <t>To do: Circuit Wizard sim sweeping 12 → 9 V to find my switch point; try R_B1 = 677 Ω vs 10 kΩ; try an LDR version (light/dark indicator).</t>
+          <t>Sim used 1N4740 (10 V) instead of BZX85C10. To do: 0.1 V sweep between 10 and 11 V to find my switch point (video ≈ 10.5 V); try an LDR version (light/dark indicator).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark ep3–ep7 as finished with simulation (not uploaded yet)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LVeNQCCauU1jD51BpjCme9
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -739,9 +739,9 @@
           <t>Designing a simple circuit (closed / open) with full calculations</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E5" s="28" t="n"/>
@@ -751,11 +751,23 @@
       <c r="I5" s="25" t="n"/>
       <c r="J5" s="25" t="n"/>
       <c r="K5" s="25" t="n"/>
-      <c r="L5" s="25" t="n"/>
+      <c r="L5" s="25" t="inlineStr">
+        <is>
+          <t>Done (files not uploaded yet)</t>
+        </is>
+      </c>
       <c r="M5" s="25" t="n"/>
-      <c r="N5" s="25" t="n"/>
+      <c r="N5" s="25" t="inlineStr">
+        <is>
+          <t>Not uploaded yet</t>
+        </is>
+      </c>
       <c r="O5" s="25" t="n"/>
-      <c r="P5" s="25" t="n"/>
+      <c r="P5" s="25" t="inlineStr">
+        <is>
+          <t>Finished with simulation. To do: add README summary + simulation files to GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="21">
       <c r="A6" s="25" t="inlineStr">
@@ -771,9 +783,9 @@
           <t>Designing a quiz board for two school teams</t>
         </is>
       </c>
-      <c r="D6" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" s="28" t="n"/>
@@ -783,11 +795,23 @@
       <c r="I6" s="25" t="n"/>
       <c r="J6" s="25" t="n"/>
       <c r="K6" s="25" t="n"/>
-      <c r="L6" s="25" t="n"/>
+      <c r="L6" s="25" t="inlineStr">
+        <is>
+          <t>Done (files not uploaded yet)</t>
+        </is>
+      </c>
       <c r="M6" s="25" t="n"/>
-      <c r="N6" s="25" t="n"/>
+      <c r="N6" s="25" t="inlineStr">
+        <is>
+          <t>Not uploaded yet</t>
+        </is>
+      </c>
       <c r="O6" s="25" t="n"/>
-      <c r="P6" s="25" t="n"/>
+      <c r="P6" s="25" t="inlineStr">
+        <is>
+          <t>Finished with simulation. To do: add README summary + simulation files to GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="21">
       <c r="A7" s="25" t="inlineStr">
@@ -803,9 +827,9 @@
           <t>Designing a large LED display board and choosing its component values</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" s="28" t="n"/>
@@ -815,11 +839,23 @@
       <c r="I7" s="25" t="n"/>
       <c r="J7" s="25" t="n"/>
       <c r="K7" s="25" t="n"/>
-      <c r="L7" s="25" t="n"/>
+      <c r="L7" s="25" t="inlineStr">
+        <is>
+          <t>Done (files not uploaded yet)</t>
+        </is>
+      </c>
       <c r="M7" s="25" t="n"/>
-      <c r="N7" s="25" t="n"/>
+      <c r="N7" s="25" t="inlineStr">
+        <is>
+          <t>Not uploaded yet</t>
+        </is>
+      </c>
       <c r="O7" s="25" t="n"/>
-      <c r="P7" s="25" t="n"/>
+      <c r="P7" s="25" t="inlineStr">
+        <is>
+          <t>Finished with simulation. To do: add README summary + simulation files to GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1" s="21">
       <c r="A8" s="25" t="inlineStr">
@@ -835,9 +871,9 @@
           <t>Designing a relay circuit for a contest where the fastest team wins</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" s="28" t="n"/>
@@ -847,11 +883,23 @@
       <c r="I8" s="25" t="n"/>
       <c r="J8" s="25" t="n"/>
       <c r="K8" s="25" t="n"/>
-      <c r="L8" s="25" t="n"/>
+      <c r="L8" s="25" t="inlineStr">
+        <is>
+          <t>Done (files not uploaded yet)</t>
+        </is>
+      </c>
       <c r="M8" s="25" t="n"/>
-      <c r="N8" s="25" t="n"/>
+      <c r="N8" s="25" t="inlineStr">
+        <is>
+          <t>Not uploaded yet</t>
+        </is>
+      </c>
       <c r="O8" s="25" t="n"/>
-      <c r="P8" s="25" t="n"/>
+      <c r="P8" s="25" t="inlineStr">
+        <is>
+          <t>Finished with simulation. To do: add README summary + simulation files to GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1" s="21">
       <c r="A9" s="25" t="inlineStr">
@@ -867,9 +915,9 @@
           <t>Designing a fish tank circuit based on sunlight intensity, with a light cell</t>
         </is>
       </c>
-      <c r="D9" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E9" s="28" t="n"/>
@@ -879,11 +927,23 @@
       <c r="I9" s="25" t="n"/>
       <c r="J9" s="25" t="n"/>
       <c r="K9" s="25" t="n"/>
-      <c r="L9" s="25" t="n"/>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>Done (files not uploaded yet)</t>
+        </is>
+      </c>
       <c r="M9" s="25" t="n"/>
-      <c r="N9" s="25" t="n"/>
+      <c r="N9" s="25" t="inlineStr">
+        <is>
+          <t>Not uploaded yet</t>
+        </is>
+      </c>
       <c r="O9" s="25" t="n"/>
-      <c r="P9" s="25" t="n"/>
+      <c r="P9" s="25" t="inlineStr">
+        <is>
+          <t>Finished with simulation. To do: add README summary + simulation files to GitHub.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="165" customHeight="1" s="21">
       <c r="A10" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Add ep11 summary: driver transistor and car cooling fan control
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -1211,7 +1211,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1" s="21">
+    <row r="13" ht="165" customHeight="1" s="21">
       <c r="A13" s="25" t="inlineStr">
         <is>
           <t>Professional Electronic Design Course</t>
@@ -1225,23 +1225,80 @@
           <t>Designing a car-factory panel to control the cooling fan</t>
         </is>
       </c>
-      <c r="D13" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E13" s="28" t="n"/>
-      <c r="F13" s="40" t="n"/>
-      <c r="G13" s="40" t="n"/>
-      <c r="H13" s="25" t="n"/>
-      <c r="I13" s="25" t="n"/>
-      <c r="J13" s="25" t="n"/>
-      <c r="K13" s="25" t="n"/>
-      <c r="L13" s="25" t="n"/>
-      <c r="M13" s="25" t="n"/>
-      <c r="N13" s="25" t="n"/>
-      <c r="O13" s="25" t="n"/>
-      <c r="P13" s="25" t="n"/>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>46321</v>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Open README</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Watch video</t>
+        </is>
+      </c>
+      <c r="H13" s="25" t="inlineStr">
+        <is>
+          <t>• Saturation: V_CE ≈ 0 → P = V_CE × I_C ≈ 0 → no heating
+• Car rule: every load grounded to the chassis, switch the positive (high) side
+• NPN above a grounded load = emitter follower, cannot saturate
+• Driver transistor: small NPN pulls a PNP base to 0 V so the PNP saturates
+• NTC thermistor in a voltage divider as a temperature switch</t>
+        </is>
+      </c>
+      <c r="I13" s="25" t="inlineStr">
+        <is>
+          <t>1. Inverting pair with load below the NPN (fails to saturate: LED 7.8 V, motor 7 V)
+2. Driver transistor: BC547 NPN drives PNP high-side switch (+ indicator LED)
+3. Alternate form: PNP drives NPN (ground-active input)
+4. Car cooling fan controller: NTC thermistor divider → BC547B → BD140 → 12 V fan</t>
+        </is>
+      </c>
+      <c r="J13" s="25" t="inlineStr">
+        <is>
+          <t>P_loss = V_CE × I_C (2 V × 1.2 A ≈ 2.4 W)
+TIP31: 1 / 0.32 W/°C ≈ 3.1 °C/W
+V_out = V_in · R2 / (R1 + R2)
+0.4 = 12 · R2 / (8 kΩ + R2) → R2 ≈ 276 Ω → 100 Ω used</t>
+        </is>
+      </c>
+      <c r="K13" s="25" t="inlineStr">
+        <is>
+          <t>BD140 (PNP, high current), BC547B (NPN), NTC thermistor (≈ 8 kΩ at 25 °C, ≈ 100 Ω hot), R2 = 100 Ω, 1 kΩ, red LED, 12 V fan, 12 V supply. Datasheets read: TIP31/32 (40 W), BC547 (500 mW), 2N2222 (2.28 mW/°C)</t>
+        </is>
+      </c>
+      <c r="L13" s="25" t="inlineStr">
+        <is>
+          <t>Not done yet</t>
+        </is>
+      </c>
+      <c r="M13" s="25" t="inlineStr">
+        <is>
+          <t>Video sim: NPN above load → LED 7.8 V, motor ≈ 7–9 V (≈ 2 V lost); PNP driver → LED 11.58 V, lamp + motor ≈ 11 V, 11.18 V at 1.5 A with 1 kΩ. Fan sim: ≈ 0.5 V cold (off), ≈ 2 V hot (on).
+Hardware: soldering iron near thermistor → red LED + fan on; removed → off. Fan aimed at the sensor turns on/off quickly.</t>
+        </is>
+      </c>
+      <c r="N13" s="25" t="inlineStr">
+        <is>
+          <t>README only (no media yet)</t>
+        </is>
+      </c>
+      <c r="O13" s="25" t="inlineStr">
+        <is>
+          <t>A grounded load needs a PNP on the high side, and a small NPN driver is what pulls it fully into saturation. Add a thermistor divider in front and the same block becomes an automatic temperature-controlled fan.</t>
+        </is>
+      </c>
+      <c r="P13" s="25" t="inlineStr">
+        <is>
+          <t>To do: Circuit Wizard sim of the fan controller (sweep temperature, log divider and fan voltage); compare V_CE / power of NPN-above-load vs PNP driver at ≈ 1.2 A; find switch-on thermistor resistance (my estimate ≈ 2 kΩ).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1" s="21">
       <c r="A14" s="25" t="inlineStr">
@@ -3374,6 +3431,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId8"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add ep11 simulation videos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016Bc4mu8GrYKXC5FPkSmyMK
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -1227,7 +1227,7 @@
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E13" s="28" t="n">
@@ -1275,7 +1275,10 @@
       </c>
       <c r="L13" s="25" t="inlineStr">
         <is>
-          <t>Not done yet</t>
+          <t>• NPN above load: V_CE = 4.20 V (LED pull-up) / 4.12 V (10 kΩ pull-up) → load 7.8 V, matches video ✔
+• Driver BC547B → TIP127: LED V_CE = 412 mV ✔; motor V_CE = 489–577 mV ✔ (≈ 10× less waste)
+• PNP drives NPN, switch to ground: output NPN V_CE = 54.85 mV ✔
+• Fan controller (10 kΩ NTC, R5 = 100 Ω): off up to 56.9 °C; starts at 2.07 kΩ / 64.6 °C (my ≈ 2 kΩ estimate ✔); at 80 °C BD140 still drops 9.05 V ✘ (not saturated)</t>
         </is>
       </c>
       <c r="M13" s="25" t="inlineStr">
@@ -1286,17 +1289,17 @@
       </c>
       <c r="N13" s="25" t="inlineStr">
         <is>
-          <t>README only (no media yet)</t>
+          <t>6 simulation GIFs + MP4s: NPN above load (LED pull-up, 10 kΩ pull-up), TIP127 driver (LED, motor), PNP→NPN ground-active input, thermistor fan controller sweep</t>
         </is>
       </c>
       <c r="O13" s="25" t="inlineStr">
         <is>
-          <t>A grounded load needs a PNP on the high side, and a small NPN driver is what pulls it fully into saturation. Add a thermistor divider in front and the same block becomes an automatic temperature-controlled fan.</t>
+          <t>A grounded load needs a PNP on the high side, and a small NPN driver is what pulls it fully into saturation. Add a thermistor divider in front and the same block becomes an automatic temperature-controlled fan. In my sim, the fan controller showed that a driver only helps if the first transistor saturates too: a &lt; 1 V divider through 10 kΩ starves Q1, so the BD140 wasted ≈ 9 V.</t>
         </is>
       </c>
       <c r="P13" s="25" t="inlineStr">
         <is>
-          <t>To do: Circuit Wizard sim of the fan controller (sweep temperature, log divider and fan voltage); compare V_CE / power of NPN-above-load vs PNP driver at ≈ 1.2 A; find switch-on thermistor resistance (my estimate ≈ 2 kΩ).</t>
+          <t>Sims used TIP127 (PNP Darlington) instead of BD140 for the switch demos, and a 10 kΩ@25 °C thermistor. To do: fix fan controller (R1 10 kΩ → ≈ 1 kΩ, R3 600 Ω → ≈ 2.2 kΩ) and re-check V_CE at 80 °C; try BD140 in the switch sims; add an ammeter to compute P = V_CE × I_fan; compare R2 = 276 Ω vs 100 Ω.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ep12 summary: RC time delays and delayed fan turn-off
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHpR46XbKVCGVpJLUPDgMg
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -1303,7 +1303,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1" s="21">
+    <row r="14" ht="165" customHeight="1" s="21">
       <c r="A14" s="25" t="inlineStr">
         <is>
           <t>Professional Electronic Design Course</t>
@@ -1317,23 +1317,84 @@
           <t>Designing a car-factory circuit for testing fans</t>
         </is>
       </c>
-      <c r="D14" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="40" t="n"/>
-      <c r="G14" s="40" t="n"/>
-      <c r="H14" s="25" t="n"/>
-      <c r="I14" s="25" t="n"/>
-      <c r="J14" s="25" t="n"/>
-      <c r="K14" s="25" t="n"/>
-      <c r="L14" s="25" t="n"/>
-      <c r="M14" s="25" t="n"/>
-      <c r="N14" s="25" t="n"/>
-      <c r="O14" s="25" t="n"/>
-      <c r="P14" s="25" t="n"/>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E14" s="28" t="n">
+        <v>46324</v>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>Open README</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="inlineStr">
+        <is>
+          <t>Watch video</t>
+        </is>
+      </c>
+      <c r="H14" s="25" t="inlineStr">
+        <is>
+          <t>• R + C in series in a DC circuit = time delay (τ = RC, ≈ 5τ to full)
+• Capacitor charged directly → delayed OFF; resistor before capacitor → delayed ON; series capacitor → self-turn-off pulse
+• Diodes (n × 0.7 V) or Zener (V_Z + 0.7 V) set a fixed threshold the capacitor must reach
+• Staircase-light timer (capacitor holds transistor + relay on)
+• Blocking diode forces the capacitor to discharge only into the transistor base
+• Delay stops the fan flickering on/off when it cools its own sensor</t>
+        </is>
+      </c>
+      <c r="I14" s="25" t="inlineStr">
+        <is>
+          <t>1. Staircase-light timer: 9 V, switch → capacitor → NPN → relay → 220 V lamp (video sim)
+2. 12 V fan, NPN→PNP high-side driver, 470 µF delayed off (hardware)
+3. Divider + 5.1 V Zener delayed on (≈ 4 s start delay, hardware)
+4. Thermistor fan controller + 470 µF + blocking diode (delayed fan turn-off)</t>
+        </is>
+      </c>
+      <c r="J14" s="25" t="inlineStr">
+        <is>
+          <t>τ = R·C
+V_C(t) = V_s(1 − e^(−t/RC)); V_C(t) = V_0·e^(−t/RC)
+Threshold = n × 0.7 V (diodes) or V_Z + 0.7 V (5.1 + 0.7 = 5.8 V)
+My sim: τ = 10 kΩ × 470 µF = 4.7 s (with diode); ≈ (1 kΩ ∥ 10 kΩ) × 500 µF ≈ 0.45 s (no diode)</t>
+        </is>
+      </c>
+      <c r="K14" s="25" t="inlineStr">
+        <is>
+          <t>BD140 (PNP), NPN driver, 470 µF timing capacitor, 10 kΩ base resistor, 1 kΩ, LED + 220 Ω, silicon blocking diode, NTC thermistor + 220 Ω (hardware) / 33 kΩ NTC + 1 kΩ (my sim), 5.1 V Zener (variation)</t>
+        </is>
+      </c>
+      <c r="L14" s="25" t="inlineStr">
+        <is>
+          <t>• With diode (470 µF): fan on in &lt; 1 s; after cooling, V_CE(Q2) climbs 8.23 → 11.46 V, LED off after ≈ 13 s, fan settled ≈ 16 s ✔ (est. ≈ 10.5 s from τ = 4.7 s)
+• Without diode (500 µF): off within ≈ 1 s ✔ (τ ≈ 0.45 s)
+• ✘ PNP not saturated when hot: V_CE 7.7–8.2 V, fan gets only ≈ 4 V (driver starved: ≈ 0.1 mA base vs ≈ 45 mA LED branch)</t>
+        </is>
+      </c>
+      <c r="M14" s="25" t="inlineStr">
+        <is>
+          <t>Video sim: 100 µF → no delay, 1000 µF without diode → ≈ 1 s; with diode → much longer
+Hardware: fan keeps running after heat removed until cap empties ✔; without capacitor the fan flickers on/off even with heat present
+Zener variation: ≈ 4 s start delay, stops almost at once</t>
+        </is>
+      </c>
+      <c r="N14" s="25" t="inlineStr">
+        <is>
+          <t>2 simulation GIFs + MP4s: fan delay with blocking diode, fan delay without diode</t>
+        </is>
+      </c>
+      <c r="O14" s="25" t="inlineStr">
+        <is>
+          <t>Adding a capacitor is not enough: check where it discharges. A blocking diode makes the charge go only into the transistor base, so the fan turns on fast but turns off slowly, which also stops it flickering.</t>
+        </is>
+      </c>
+      <c r="P14" s="25" t="inlineStr">
+        <is>
+          <t>Sim used Circuit Wizard 33 kΩ NTC with 1 kΩ bottom resistor (video: ≈ 8 kΩ NTC + 220 Ω). To do: raise LED resistor to ≈ 2.2 kΩ so Q1/Q2 saturate; try 1000 µF / 22 kΩ; build the Zener delayed-on variation.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1" s="21">
       <c r="A15" s="25" t="inlineStr">
@@ -3436,6 +3497,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId10"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add ep13 summary: useless machine motor circuit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHpR46yMNJVEUaEQH7jgS4
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -1396,7 +1396,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" s="21">
+    <row r="15" ht="165" customHeight="1" s="21">
       <c r="A15" s="25" t="inlineStr">
         <is>
           <t>Professional Electronic Design Course</t>
@@ -1410,23 +1410,84 @@
           <t>Designing a useless machine motor circuit</t>
         </is>
       </c>
-      <c r="D15" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E15" s="28" t="n"/>
-      <c r="F15" s="40" t="n"/>
-      <c r="G15" s="40" t="n"/>
-      <c r="H15" s="25" t="n"/>
-      <c r="I15" s="25" t="n"/>
-      <c r="J15" s="25" t="n"/>
-      <c r="K15" s="25" t="n"/>
-      <c r="L15" s="25" t="n"/>
-      <c r="M15" s="25" t="n"/>
-      <c r="N15" s="25" t="n"/>
-      <c r="O15" s="25" t="n"/>
-      <c r="P15" s="25" t="n"/>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>Open README</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Watch video</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="inlineStr">
+        <is>
+          <t>• Ground = the point the designer calls 0 V; all ground symbols are one node
+• Voltage of a node depends on the reference (3 / 6 / 9 / 12 V on a 4-resistor divider)
+• Zener + transistor branch needs the tap ≈ V_Z + 0.7 V above the emitter
+• Two batteries in series, midpoint grounded → ± supply (capacitor split fails under load)
+• Complementary NPN/PNP pair steers +V or −V to a motor → direction control
+• NC limit switch in the −V (return) line stops the motor at home</t>
+        </is>
+      </c>
+      <c r="I15" s="25" t="inlineStr">
+        <is>
+          <t>1. 4 × 1 kΩ divider on 12 V, voltmeter reference moved (my sim)
+2. Divider tap → Zener → NPN → LED, ground position moved (video + my sim)
+3. ± supply: two batteries vs. two capacitors (video sim)
+4. Useless machine: ± supply, SPDT switch, 1 kΩ → BC547/BD140 pair, motor, direction LEDs, NC limit switch</t>
+        </is>
+      </c>
+      <c r="J15" s="25" t="inlineStr">
+        <is>
+          <t>V_R = 12 V / 4 = 3 V each
+V_on ≈ V_Z + V_BE (+ I_B·R_B)
+V_th = V·R_bottom/(R_top+R_bottom), R_th = R_top ∥ R_bottom
+V_motor ≈ ±(V_s − 0.7 V)
+I_LED ≈ (8.3 − 2) / 220 ≈ 29 mA</t>
+        </is>
+      </c>
+      <c r="K15" s="25" t="inlineStr">
+        <is>
+          <t>BC547 (NPN), BD140 (PNP), 1 kΩ base resistor, 2 batteries (± supply), small 5 V motor + 3 × 100 Ω ∥ series dropper, ON-ON toggle (SPDT), lever micro switch (COM + NC), red + green LEDs with resistors. My sim: ±9 V, 220 Ω LED resistors, 1N751 5.1 V Zener</t>
+        </is>
+      </c>
+      <c r="L15" s="25" t="inlineStr">
+        <is>
+          <t>• Voltmeter on divider: 3.00 / 12.00 / 9.00 / 6.00 V ✔ (exactly 3 V per resistor)
+• Zener LED branch: on with tap 9 V above ground (tap loaded to 7.66 V, I_B ≈ 1.79 mA → V_Z ≈ 5.2 V); off at 3 V and 6 V (needs ≈ 5.8 V, R_th ≈ 667 Ω); on again with D1 moved to top rail
+• Useless machine (±9 V): SW1 up → D1 + forward ✔; down → D2 + reverse ✔; SW2 open → stop ✔</t>
+        </is>
+      </c>
+      <c r="M15" s="25" t="inlineStr">
+        <is>
+          <t>Video sim: tap 3 V → LED off, 6 V → on (3.9 V Zener); with 1.5 V battery in emitter path, 6 V → off, 9 V → on. Capacitor split: ±6 V unloaded, collapses to 0 / −12 V with a 1 kΩ load.
+Hardware: press → red (arm flips switch off) → green (returns) → off at home; works even if re-pressed halfway.</t>
+        </is>
+      </c>
+      <c r="N15" s="25" t="inlineStr">
+        <is>
+          <t>3 simulation GIFs + MP4s: ground reference divider, ground position vs. Zener LED, useless machine with limit switch</t>
+        </is>
+      </c>
+      <c r="O15" s="25" t="inlineStr">
+        <is>
+          <t>Ground is only a reference I choose. A complementary pair lets one signal choose + or − for a motor, and one normally closed switch in the right line (the −V return path only) turns it into a useless machine that stops itself.</t>
+        </is>
+      </c>
+      <c r="P15" s="25" t="inlineStr">
+        <is>
+          <t>Video link: only the playlist is linked; replace with the direct ep13 URL. No .cwz files sent yet. To do: save circuits as .cwz, measure motor voltage, LED resistors → 330 Ω, try 3.9 V Zener in sim 2, simulate capacitor split.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1" s="21">
       <c r="A16" s="25" t="inlineStr">
@@ -3499,6 +3560,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId12"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add ep13 Circuit Wizard files and video link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHpR46yMNJVEUaEQH7jgS4
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -1475,7 +1475,8 @@
       </c>
       <c r="N15" s="25" t="inlineStr">
         <is>
-          <t>3 simulation GIFs + MP4s: ground reference divider, ground position vs. Zener LED, useless machine with limit switch</t>
+          <t>3 simulation GIFs + MP4s: ground reference divider, ground position vs. Zener LED, useless machine with limit switch
+3 circuit files (.cwz): useless machine (final), motor reversing pair (starting circuit), ground position Zener LED</t>
         </is>
       </c>
       <c r="O15" s="25" t="inlineStr">
@@ -1485,7 +1486,7 @@
       </c>
       <c r="P15" s="25" t="inlineStr">
         <is>
-          <t>Video link: only the playlist is linked; replace with the direct ep13 URL. No .cwz files sent yet. To do: save circuits as .cwz, measure motor voltage, LED resistors → 330 Ω, try 3.9 V Zener in sim 2, simulate capacitor split.</t>
+          <t>Sim motor is Circuit Wizard "DC Motor (3V DC)" fed ≈ 8.3 V. To do: add a series dropper resistor for the motor, measure motor voltage, LED resistors → 330 Ω, try 3.9 V Zener in sim 2, simulate capacitor split.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ep14 summary and Circuit Wizard file: secret-code circuit
- New folder ep14-secret-code-circuit-no-programming with English summary
  (4-step design, MOSFET gate pull-down, 10 kOhm short protection,
  BJT vs MOSFET comparison) and the .cwz circuit file
- Course index: ep14 done, Level 2 in progress
- Main README: 14 / 77
- Episode index spreadsheet: ep14 row filled in

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHpR467HqXo1BKfEYWGVRS
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -1490,7 +1490,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1" s="21">
+    <row r="16" ht="165" customHeight="1" s="21">
       <c r="A16" s="25" t="inlineStr">
         <is>
           <t>Professional Electronic Design Course</t>
@@ -1504,23 +1504,83 @@
           <t>Designing a secret-code circuit without programming</t>
         </is>
       </c>
-      <c r="D16" s="26" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E16" s="28" t="n"/>
-      <c r="F16" s="40" t="n"/>
-      <c r="G16" s="40" t="n"/>
-      <c r="H16" s="25" t="n"/>
-      <c r="I16" s="25" t="n"/>
-      <c r="J16" s="25" t="n"/>
-      <c r="K16" s="25" t="n"/>
-      <c r="L16" s="25" t="n"/>
-      <c r="M16" s="25" t="n"/>
-      <c r="N16" s="25" t="n"/>
-      <c r="O16" s="25" t="n"/>
-      <c r="P16" s="25" t="n"/>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E16" s="28" t="n">
+        <v>46326</v>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Open README</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>Watch video</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="inlineStr">
+        <is>
+          <t>• Level 2 intro: circuits that decide on/off by themselves, no programming
+• Switches in series = AND (all must be closed); parallel = OR
+• Wrong switches must actively veto: pull the MOSFET gate to 0 V
+• Pulling a supplied node to ground = battery short → series resistor fixes it
+• MOSFET gate is a capacitor → gate pull-down (10 kΩ–1 MΩ)
+• BJT vs. MOSFET: switching speed, power loss, input drive voltage</t>
+        </is>
+      </c>
+      <c r="I16" s="25" t="inlineStr">
+        <is>
+          <t>1. Correct switches 4-5-6-8 in series straight to the solenoid (extra switches ignored ✘)
+2. Series chain → N-MOSFET gate, low-side switch, gate pull-down
+3. Wrong switches ground the gate (works, but shorts the battery ✘)
+4. 10 kΩ series resistor before the gate (final design ✔)
+5. Variants: NPN base version; DIP switch + relay version (code 1-3-6)</t>
+        </is>
+      </c>
+      <c r="J16" s="25" t="inlineStr">
+        <is>
+          <t>V_G = 12 × 10k / (10k + 10k) = 6 V
+I_short = 12 V / 10 kΩ = 1.2 mA
+P_BJT = V_CE(sat) × I_C = 0.6 × 0.1 = 60 mW
+P_MOSFET = I_D² × R_DS(on) = 0.1² × 5 = 50 mW</t>
+        </is>
+      </c>
+      <c r="K16" s="25" t="inlineStr">
+        <is>
+          <t>2N7000 N-MOSFET (R_DS(on) ≈ 5 Ω, I_D ≈ 200 mA, V_GS(th) 0.8–3 V), 2 × 10 kΩ (series + gate pull-down), 12 V solenoid lock, flyback diode across the solenoid, 10 latching switches (0–9), 12 V supply. Compared: BC547B (V_CE(sat) 0.2–0.6 V, 100 mA)</t>
+        </is>
+      </c>
+      <c r="L16" s="25" t="inlineStr">
+        <is>
+          <t>Circuit file only (no recording yet): 12 V, ideal N-MOSFET, 6 V DC solenoid, 2 × 10 kΩ, 10 SPST switches. Expected: 4-5-6-8 → gate ≈ 6 V, solenoid on; any extra switch → gate ≈ 0 V, ≈ 1.2 mA</t>
+        </is>
+      </c>
+      <c r="M16" s="25" t="inlineStr">
+        <is>
+          <t>4 → 5 → 6 → 8 → MOSFET on, solenoid pulls in ✔
+Adding 7, 0 or 1 → releases at once ✔
+0, 5, 6, 8 (no 4) → stays locked ✔</t>
+        </is>
+      </c>
+      <c r="N16" s="25" t="inlineStr">
+        <is>
+          <t>1 circuit file (.cwz): secret-code lock (final design)</t>
+        </is>
+      </c>
+      <c r="O16" s="25" t="inlineStr">
+        <is>
+          <t>Series switches make an AND, but a lock must also reject extra inputs: wrong switches pull the gate to 0 V, and one 10 kΩ resistor stops that from shorting the battery. For a 12 V, 100 mA lock a BJT and a MOSFET are equivalent (≈ 60 vs. 50 mW).</t>
+        </is>
+      </c>
+      <c r="P16" s="25" t="inlineStr">
+        <is>
+          <t>Sim uses Circuit Wizard "Solenoid (6V DC)" on 12 V and has no flyback diode. To do: record simulation, measure gate voltage (≈ 6 V) and series-resistor current (≈ 1.2 mA); try without the 10 kΩ / without the pull-down; BC547B version.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="21">
       <c r="A17" s="25" t="inlineStr">
@@ -3563,6 +3623,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId14"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add ep14 simulation video
- media/ep14-sim-secret-code-lock.gif (1.5x, cropped) + original MP4
- README: simulation section with wiring, recorded timeline and results
- Course index and episode index spreadsheet updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHpR467HqXo1BKfEYWGVRS
</commit_message>
<xml_diff>
--- a/Electricity-Diploma-Episode-Index.xlsx
+++ b/Electricity-Diploma-Episode-Index.xlsx
@@ -1556,7 +1556,12 @@
       </c>
       <c r="L16" s="25" t="inlineStr">
         <is>
-          <t>Circuit file only (no recording yet): 12 V, ideal N-MOSFET, 6 V DC solenoid, 2 × 10 kΩ, 10 SPST switches. Expected: 4-5-6-8 → gate ≈ 6 V, solenoid on; any extra switch → gate ≈ 0 V, ≈ 1.2 mA</t>
+          <t>Code SW4, SW5, SW6, SW8 (SW1–SW10 = digits 1–9, 0), R2 = 10 kΩ series, R1 = 10 kΩ pull-down, ideal N-MOSFET, 6 V solenoid on 12 V:
+• Code only → gate high, solenoid pulled in ✔
+• SW4 opened → gate 0 V, released ✔
+• Code + wrong switch → chain at 12 V up to R2, gate 0 V, released, no short ✔
+• Wrong switch opened → pulled in again ✔
+(No meters: V_G ≈ 6 V and 1.2 mA are calculated)</t>
         </is>
       </c>
       <c r="M16" s="25" t="inlineStr">
@@ -1568,7 +1573,8 @@
       </c>
       <c r="N16" s="25" t="inlineStr">
         <is>
-          <t>1 circuit file (.cwz): secret-code lock (final design)</t>
+          <t>1 simulation GIF + MP4: secret-code lock (code on, code broken, code + wrong switch)
+1 circuit file (.cwz): secret-code lock (final design)</t>
         </is>
       </c>
       <c r="O16" s="25" t="inlineStr">
@@ -1578,7 +1584,7 @@
       </c>
       <c r="P16" s="25" t="inlineStr">
         <is>
-          <t>Sim uses Circuit Wizard "Solenoid (6V DC)" on 12 V and has no flyback diode. To do: record simulation, measure gate voltage (≈ 6 V) and series-resistor current (≈ 1.2 mA); try without the 10 kΩ / without the pull-down; BC547B version.</t>
+          <t>Sim uses Circuit Wizard "Solenoid (6V DC)" on 12 V and has no flyback diode. To do: add a gate voltmeter (≈ 6 V) and an ammeter on R2 (≈ 1.2 mA); try without R2 / without the pull-down; BC547B version.</t>
         </is>
       </c>
     </row>

</xml_diff>